<commit_message>
Update team.xlsx: add pro riders
</commit_message>
<xml_diff>
--- a/team.xlsx
+++ b/team.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unilever-my.sharepoint.com/personal/karol_borowiak_unilever_com/Documents/Desktop/progr/zwiftpower profile update/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloud\zwiftpower-excel-updater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{060829F7-0A24-4757-B053-FCC45D23A1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{532C3F2D-BB87-4061-AD07-1E45A7F13F13}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54BAF0DC-A49B-4130-9BFB-712D1C177CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5835" yWindow="3360" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dane_zawodnika" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Imię i nazwisko</t>
   </si>
@@ -46,6 +46,21 @@
   </si>
   <si>
     <t>Karol Borowiak</t>
+  </si>
+  <si>
+    <t>Adrien Legriffon</t>
+  </si>
+  <si>
+    <t>Njal Pedersen</t>
+  </si>
+  <si>
+    <t>Philippe Legros</t>
+  </si>
+  <si>
+    <t>Ed Laverack</t>
+  </si>
+  <si>
+    <t>Ruben Dhondt</t>
   </si>
 </sst>
 </file>
@@ -101,7 +116,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -119,7 +134,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Pakiet Office 2007–2010">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -157,7 +172,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Pakiet Office 2007–2010">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -229,7 +244,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Pakiet Office 2007–2010">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -403,14 +418,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -418,12 +433,52 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>4273591</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>627192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>3201227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5296096</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>703388</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>2230709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>